<commit_message>
Seed verified US skincare sources
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Videos" sheetId="1" r:id="Rf35fd4d4eebd4666"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rdb0e7dbff4504d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="3" r:id="R38c05541158548a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric History" sheetId="4" r:id="R3fbf9f0ac3e44ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Relevance" sheetId="5" r:id="Red2ffd23975e4f9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated Briefs" sheetId="6" r:id="R7ddde0fb09854b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="Ra374857476f84645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Rc9f0bcdeda7f4d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top Videos" sheetId="1" r:id="R8a11f2b2af844942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rc5adf856d41d46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="3" r:id="R23558e8765b542a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric History" sheetId="4" r:id="Re51144e1bf984e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Relevance" sheetId="5" r:id="R431bc2ec52514f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated Briefs" sheetId="6" r:id="R5fd6f3554e2945c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="Rca512817bdac452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="R4f86e3fbd0064fb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -355,7 +355,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Generated 2026-09-07T04:50:26+00:00. Demo fixture data — not live trend evidence.</x:v>
+        <x:v>Generated 2026-09-07T05:09:12+00:00. Verified source data.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -405,134 +405,268 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="n">
-        <x:v>61.66</x:v>
+        <x:v>51.02</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>Fixture UGC Creator</x:v>
+        <x:v>Joyce Kim, MD Dermatologist</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_creator/video/7000000000000000002</x:v>
+        <x:v>https://www.tiktok.com/@dermlifebalance/video/7237931605216464171</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>worth the hype</x:v>
+        <x:v>brutally honest review</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>talking head</x:v>
+        <x:v>expert review</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
-        <x:v>A 30-day test answers whether a viral moisturizer deserves the hype.</x:v>
-      </x:c>
-      <x:c r="G5" s="3" t="n">
-        <x:v>420000</x:v>
-      </x:c>
+        <x:v>A dermatologist gives a non-sponsored verdict after ten months of use.</x:v>
+      </x:c>
+      <x:c r="G5" s="3"/>
       <x:c r="H5" s="3" t="n">
-        <x:v>39000</x:v>
-      </x:c>
-      <x:c r="I5" s="3" t="n">
-        <x:v>980</x:v>
-      </x:c>
-      <x:c r="J5" s="3" t="n">
-        <x:v>4100</x:v>
-      </x:c>
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="I5" s="3"/>
+      <x:c r="J5" s="3"/>
       <x:c r="K5" s="3" t="str">
-        <x:v>2026-09-07 05:00</x:v>
+        <x:v>2026-09-07 05:09</x:v>
       </x:c>
       <x:c r="L5" s="3" t="str">
-        <x:v>measured</x:v>
+        <x:v>insufficient_history</x:v>
       </x:c>
       <x:c r="M5" s="3" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="N5" s="3" t="str">
-        <x:v>fixture</x:v>
+        <x:v>medium</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="n">
-        <x:v>61.25</x:v>
+        <x:v>48.15</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>Fixture Dermatologist</x:v>
+        <x:v>Michael Park, MD</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_derm/video/7000000000000000001</x:v>
+        <x:v>https://www.tiktok.com/@dr.michaelpark10/video/7615984815053098254</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>dermatologist rates</x:v>
+        <x:v>affordable alternative</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
-        <x:v>expert review</x:v>
+        <x:v>talking head</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>A dermatologist ranks five viral barrier serums from worst to best.</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="n">
-        <x:v>840000</x:v>
-      </x:c>
+        <x:v>A surprising two-dollar price reframes an expert-recommended cleanser.</x:v>
+      </x:c>
+      <x:c r="G6" s="3"/>
       <x:c r="H6" s="3" t="n">
-        <x:v>72000</x:v>
-      </x:c>
-      <x:c r="I6" s="3" t="n">
-        <x:v>2100</x:v>
-      </x:c>
-      <x:c r="J6" s="3" t="n">
-        <x:v>8900</x:v>
-      </x:c>
+        <x:v>3920</x:v>
+      </x:c>
+      <x:c r="I6" s="3"/>
+      <x:c r="J6" s="3"/>
       <x:c r="K6" s="3" t="str">
-        <x:v>2026-09-07 05:00</x:v>
+        <x:v>2026-09-07 05:09</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str">
-        <x:v>measured</x:v>
+        <x:v>insufficient_history</x:v>
       </x:c>
       <x:c r="M6" s="3" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="N6" s="3" t="str">
-        <x:v>fixture</x:v>
+        <x:v>medium</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="n">
-        <x:v>61.14</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="str">
-        <x:v>Fixture Esthetician</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="str">
-        <x:v>https://www.tiktok.com/@fixture_esthetician/video/7000000000000000003</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="str">
+      <x:c r="A7" s="3" t="n">
+        <x:v>46.36</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>Dr. Jing (Jenny) Liu</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drjennyliu/video/7587041392862563598</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="str">
+        <x:v>dermatologist rates</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="str">
+        <x:v>ranking</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="str">
+        <x:v>A dermatologist rapidly rates viral Korean skincare products.</x:v>
+      </x:c>
+      <x:c r="G7" s="3"/>
+      <x:c r="H7" s="3" t="n">
+        <x:v>31200</x:v>
+      </x:c>
+      <x:c r="I7" s="3"/>
+      <x:c r="J7" s="3"/>
+      <x:c r="K7" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="L7" s="3" t="str">
+        <x:v>insufficient_history</x:v>
+      </x:c>
+      <x:c r="M7" s="3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N7" s="3" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="n">
+        <x:v>45.57</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Dr. Daniel Sugai</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drspf/video/7580106279092342047</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>products I trust</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>expert review</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>A dermatologist names the facial moisturizers he considers best.</x:v>
+      </x:c>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3" t="n">
+        <x:v>7672</x:v>
+      </x:c>
+      <x:c r="I8" s="3"/>
+      <x:c r="J8" s="3"/>
+      <x:c r="K8" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="L8" s="3" t="str">
+        <x:v>insufficient_history</x:v>
+      </x:c>
+      <x:c r="M8" s="3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N8" s="3" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="n">
+        <x:v>45.51</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>Dr Dray | Dermatologist</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drdrayzday/video/7576419565450628365</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="str">
+        <x:v>dermatologist rates</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="str">
+        <x:v>expert review</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="str">
+        <x:v>A dermatologist reviews a widely discussed Medicube product.</x:v>
+      </x:c>
+      <x:c r="G9" s="3"/>
+      <x:c r="H9" s="3" t="n">
+        <x:v>19400</x:v>
+      </x:c>
+      <x:c r="I9" s="3"/>
+      <x:c r="J9" s="3"/>
+      <x:c r="K9" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="L9" s="3" t="str">
+        <x:v>insufficient_history</x:v>
+      </x:c>
+      <x:c r="M9" s="3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N9" s="3" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="n">
+        <x:v>44.05</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>elevenesthetician</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>https://www.tiktok.com/@elevenesthetician/video/7563054629290790199</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
         <x:v>best vs worst</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="str">
+      <x:c r="E10" s="3" t="str">
         <x:v>ranking</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="str">
-        <x:v>An esthetician names the best and worst drugstore cleansers.</x:v>
-      </x:c>
-      <x:c r="G7" s="4" t="n">
-        <x:v>1250000</x:v>
-      </x:c>
-      <x:c r="H7" s="4" t="n">
-        <x:v>115000</x:v>
-      </x:c>
-      <x:c r="I7" s="4" t="n">
-        <x:v>3600</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="n">
-        <x:v>17200</x:v>
-      </x:c>
-      <x:c r="K7" s="4" t="str">
-        <x:v>2026-09-07 05:00</x:v>
-      </x:c>
-      <x:c r="L7" s="4" t="str">
-        <x:v>measured</x:v>
-      </x:c>
-      <x:c r="M7" s="4" t="n">
+      <x:c r="F10" s="3" t="str">
+        <x:v>An esthetician separates one brand's best products from its worst.</x:v>
+      </x:c>
+      <x:c r="G10" s="3"/>
+      <x:c r="H10" s="3" t="n">
+        <x:v>3226</x:v>
+      </x:c>
+      <x:c r="I10" s="3"/>
+      <x:c r="J10" s="3"/>
+      <x:c r="K10" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="L10" s="3" t="str">
+        <x:v>insufficient_history</x:v>
+      </x:c>
+      <x:c r="M10" s="3" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="N7" s="4" t="str">
-        <x:v>fixture</x:v>
+      <x:c r="N10" s="3" t="str">
+        <x:v>high</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="4" t="n">
+        <x:v>42.4</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Angela Park</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>https://www.tiktok.com/@angelaypark/video/7627631712436030750</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>products I trust</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="str">
+        <x:v>talking head</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>A creator names trusted Sephora products and anchors recommendations in her skin type.</x:v>
+      </x:c>
+      <x:c r="G11" s="4"/>
+      <x:c r="H11" s="4" t="n">
+        <x:v>2163</x:v>
+      </x:c>
+      <x:c r="I11" s="4"/>
+      <x:c r="J11" s="4"/>
+      <x:c r="K11" s="4" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="L11" s="4" t="str">
+        <x:v>insufficient_history</x:v>
+      </x:c>
+      <x:c r="M11" s="4" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="N11" s="4" t="str">
+        <x:v>medium</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -593,53 +727,87 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>worth the hype</x:v>
+        <x:v>brutally honest review</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="3" t="n">
-        <x:v>61.66</x:v>
+        <x:v>51.02</x:v>
       </x:c>
       <x:c r="D5" s="3" t="n">
-        <x:v>61.66</x:v>
+        <x:v>51.02</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_creator/video/7000000000000000002</x:v>
+        <x:v>https://www.tiktok.com/@dermlifebalance/video/7237931605216464171</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>dermatologist rates</x:v>
+        <x:v>affordable alternative</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="3" t="n">
-        <x:v>61.25</x:v>
+        <x:v>48.15</x:v>
       </x:c>
       <x:c r="D6" s="3" t="n">
-        <x:v>61.25</x:v>
+        <x:v>48.15</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_derm/video/7000000000000000001</x:v>
+        <x:v>https://www.tiktok.com/@dr.michaelpark10/video/7615984815053098254</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="str">
+      <x:c r="A7" s="3" t="str">
+        <x:v>dermatologist rates</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="n">
+        <x:v>45.94</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="n">
+        <x:v>46.36</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drjennyliu/video/7587041392862563598</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>products I trust</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="n">
+        <x:v>43.98</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="n">
+        <x:v>45.57</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drspf/video/7580106279092342047</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="4" t="str">
         <x:v>best vs worst</x:v>
       </x:c>
-      <x:c r="B7" s="4" t="n">
+      <x:c r="B9" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="4" t="n">
-        <x:v>61.14</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="n">
-        <x:v>61.14</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="str">
-        <x:v>https://www.tiktok.com/@fixture_esthetician/video/7000000000000000003</x:v>
+      <x:c r="C9" s="4" t="n">
+        <x:v>44.05</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="n">
+        <x:v>44.05</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="str">
+        <x:v>https://www.tiktok.com/@elevenesthetician/video/7563054629290790199</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -682,7 +850,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="31.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="9.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="45" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="5.329999923706055" hidden="0" customWidth="1"/>
@@ -718,16 +886,16 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>Fixture UGC Creator</x:v>
+        <x:v>Joyce Kim, MD Dermatologist</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>@fixture_creator</x:v>
+        <x:v>@dermlifebalance</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>Synthetic fixture profile</x:v>
+        <x:v>https://www.tiktok.com/@dermlifebalance</x:v>
       </x:c>
       <x:c r="E5" s="3" t="n">
         <x:v>1</x:v>
@@ -735,35 +903,103 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>Fixture Dermatologist</x:v>
+        <x:v>Michael Park, MD</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>@fixture_derm</x:v>
+        <x:v>@dr.michaelpark10</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>Synthetic fixture profile</x:v>
+        <x:v>https://www.tiktok.com/@dr.michaelpark10</x:v>
       </x:c>
       <x:c r="E6" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="str">
-        <x:v>Fixture Esthetician</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="str">
-        <x:v>@fixture_esthetician</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="str">
+      <x:c r="A7" s="3" t="str">
+        <x:v>Dr. Jing (Jenny) Liu</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>@drjennyliu</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="str">
-        <x:v>Synthetic fixture profile</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="n">
+      <x:c r="D7" s="3" t="str">
+        <x:v>https://www.imcas.com/en/profile/dr-jenny-jing-liu</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>Dr. Daniel Sugai</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>@drspf</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>https://www.sugaiacademy.com/about</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>Dr Dray | Dermatologist</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>@drdrayzday</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="str">
+        <x:v>https://www.drdrayzday.com/about</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>elevenesthetician</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>@elevenesthetician</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>https://www.natalierosebeauty.com/the-team</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>Angela Park</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>@angelaypark</x:v>
+      </x:c>
+      <x:c r="C11" s="4" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="str">
+        <x:v>https://thesmudgereport.com/meet-the-peoples-princesses-of-beautytok/</x:v>
+      </x:c>
+      <x:c r="E11" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -778,12 +1014,12 @@
   <x:cols>
     <x:col min="1" max="1" width="52.220001220703125" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="8.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="5.440000057220459" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="7.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="5.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="8.4399995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -830,80 +1066,128 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>7000000000000000002</x:v>
+        <x:v>7237931605216464171</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>2026-09-07 05:00</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="n">
-        <x:v>420000</x:v>
-      </x:c>
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C5" s="3"/>
       <x:c r="D5" s="3" t="n">
-        <x:v>39000</x:v>
-      </x:c>
-      <x:c r="E5" s="3" t="n">
-        <x:v>980</x:v>
-      </x:c>
-      <x:c r="F5" s="3" t="n">
-        <x:v>4100</x:v>
-      </x:c>
-      <x:c r="G5" s="3" t="n">
-        <x:v>96000</x:v>
-      </x:c>
+        <x:v>24000</x:v>
+      </x:c>
+      <x:c r="E5" s="3"/>
+      <x:c r="F5" s="3"/>
+      <x:c r="G5" s="3"/>
       <x:c r="H5" s="3" t="str">
-        <x:v>fixture</x:v>
+        <x:v>manual_csv</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>7000000000000000001</x:v>
+        <x:v>7615984815053098254</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>2026-09-07 05:00</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="n">
-        <x:v>840000</x:v>
-      </x:c>
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C6" s="3"/>
       <x:c r="D6" s="3" t="n">
-        <x:v>72000</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="n">
-        <x:v>2100</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="n">
-        <x:v>8900</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="n">
-        <x:v>310000</x:v>
-      </x:c>
+        <x:v>3920</x:v>
+      </x:c>
+      <x:c r="E6" s="3"/>
+      <x:c r="F6" s="3"/>
+      <x:c r="G6" s="3"/>
       <x:c r="H6" s="3" t="str">
-        <x:v>fixture</x:v>
+        <x:v>manual_csv</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="str">
-        <x:v>7000000000000000003</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="str">
-        <x:v>2026-09-07 05:00</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="n">
-        <x:v>1250000</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="n">
-        <x:v>115000</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="n">
-        <x:v>3600</x:v>
-      </x:c>
-      <x:c r="F7" s="4" t="n">
-        <x:v>17200</x:v>
-      </x:c>
-      <x:c r="G7" s="4" t="n">
-        <x:v>520000</x:v>
-      </x:c>
-      <x:c r="H7" s="4" t="str">
-        <x:v>fixture</x:v>
+      <x:c r="A7" s="3" t="str">
+        <x:v>7587041392862563598</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C7" s="3"/>
+      <x:c r="D7" s="3" t="n">
+        <x:v>31200</x:v>
+      </x:c>
+      <x:c r="E7" s="3"/>
+      <x:c r="F7" s="3"/>
+      <x:c r="G7" s="3"/>
+      <x:c r="H7" s="3" t="str">
+        <x:v>manual_csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>7580106279092342047</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C8" s="3"/>
+      <x:c r="D8" s="3" t="n">
+        <x:v>7672</x:v>
+      </x:c>
+      <x:c r="E8" s="3"/>
+      <x:c r="F8" s="3"/>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3" t="str">
+        <x:v>manual_csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>7576419565450628365</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C9" s="3"/>
+      <x:c r="D9" s="3" t="n">
+        <x:v>19400</x:v>
+      </x:c>
+      <x:c r="E9" s="3"/>
+      <x:c r="F9" s="3"/>
+      <x:c r="G9" s="3"/>
+      <x:c r="H9" s="3" t="str">
+        <x:v>manual_csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>7563054629290790199</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C10" s="3"/>
+      <x:c r="D10" s="3" t="n">
+        <x:v>3226</x:v>
+      </x:c>
+      <x:c r="E10" s="3"/>
+      <x:c r="F10" s="3"/>
+      <x:c r="G10" s="3"/>
+      <x:c r="H10" s="3" t="str">
+        <x:v>manual_csv</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>7627631712436030750</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>2026-09-07 05:09</x:v>
+      </x:c>
+      <x:c r="C11" s="4"/>
+      <x:c r="D11" s="4" t="n">
+        <x:v>2163</x:v>
+      </x:c>
+      <x:c r="E11" s="4"/>
+      <x:c r="F11" s="4"/>
+      <x:c r="G11" s="4"/>
+      <x:c r="H11" s="4" t="str">
+        <x:v>manual_csv</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -918,7 +1202,7 @@
     <x:col min="1" max="1" width="45" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.559999942779541" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -948,44 +1232,72 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>worth the hype</x:v>
+        <x:v>brutally honest review</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_creator/video/7000000000000000002</x:v>
+        <x:v>https://www.tiktok.com/@dermlifebalance/video/7237931605216464171</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
-        <x:v>Demo only</x:v>
+        <x:v>Review</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>dermatologist rates</x:v>
+        <x:v>affordable alternative</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
-        <x:v>https://www.tiktok.com/@fixture_derm/video/7000000000000000001</x:v>
+        <x:v>https://www.tiktok.com/@dr.michaelpark10/video/7615984815053098254</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>Demo only</x:v>
+        <x:v>Review</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="str">
+      <x:c r="A7" s="3" t="str">
+        <x:v>dermatologist rates</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drjennyliu/video/7587041392862563598</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>products I trust</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>https://www.tiktok.com/@drspf/video/7580106279092342047</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="4" t="str">
         <x:v>best vs worst</x:v>
       </x:c>
-      <x:c r="B7" s="4" t="n">
+      <x:c r="B9" s="4" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C7" s="4" t="str">
-        <x:v>https://www.tiktok.com/@fixture_esthetician/video/7000000000000000003</x:v>
-      </x:c>
-      <x:c r="D7" s="4" t="str">
-        <x:v>Demo only</x:v>
+      <x:c r="C9" s="4" t="str">
+        <x:v>https://www.tiktok.com/@elevenesthetician/video/7563054629290790199</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>Review</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1085,7 +1397,7 @@
         <x:v>Fixture records</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
         <x:v>Replace with verified live/manual sources</x:v>
@@ -1096,7 +1408,7 @@
         <x:v>Missing views</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="3" t="str">
         <x:v>Collect a new metric snapshot</x:v>
@@ -1118,7 +1430,7 @@
         <x:v>Low evidence</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
         <x:v>Human verification required</x:v>
@@ -1161,7 +1473,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
-        <x:v>46272.201689814814</x:v>
+        <x:v>46272.21472222222</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1169,7 +1481,7 @@
         <x:v>Video count</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1177,7 +1489,7 @@
         <x:v>Fixture only</x:v>
       </x:c>
       <x:c r="B7" s="11" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Teach brief builder CoBa creator format
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rbd953be22824441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rc4a2f8758fac4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R4cd897601046499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="R33f8df34bc984e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Re9c0bacf62294780"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R3ded030e06614ebd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="Rcecb5a4483fe4ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Raa1e3d279aae4617"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R85834eb203d640e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R2e83974536234e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R4d15508adc4f4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="R460d78ca5e3b4207"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Rf483f66fe11c4a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R2f41edcf21b5448c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="Rab545f1f3cdd4347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="R6227709f74aa4fdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T11:36:29+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T11:47:01+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2317,7 +2317,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>46272.483668981484</x:v>
+        <x:v>46272.4909837963</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Modernize radar and campaign brief builder
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R85834eb203d640e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R2e83974536234e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R4d15508adc4f4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="R460d78ca5e3b4207"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Rf483f66fe11c4a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R2f41edcf21b5448c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="Rab545f1f3cdd4347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="R6227709f74aa4fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R022ee2cdf4d54312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R5e99987580df4b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rac91c585bfd24f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="R4ad2030844f74f5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Rd313f82887304e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R2bcd2b6530aa4e87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R3e5134b09dfa4b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Rc71d3a636d1149ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T11:47:01+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T11:53:24+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2317,7 +2317,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>46272.4909837963</x:v>
+        <x:v>46272.495416666665</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Support dashboard opened directly from local file
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R022ee2cdf4d54312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R5e99987580df4b94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rac91c585bfd24f18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="R4ad2030844f74f5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Rd313f82887304e84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R2bcd2b6530aa4e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R3e5134b09dfa4b88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Rc71d3a636d1149ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R669bc83277cc4240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rae26f9ce099f4f7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R46b5263d83ad4a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rd4e3c57f98b74247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="R85d4f19bb66e4dd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R3608176449fd4bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R55ef157f2b1842e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Rb7cb8cb503284a05"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T11:53:24+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T12:31:56+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2317,7 +2317,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>46272.495416666665</x:v>
+        <x:v>46272.52217592593</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Add all three CoBa gifting products
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R669bc83277cc4240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rae26f9ce099f4f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R46b5263d83ad4a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rd4e3c57f98b74247"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="R85d4f19bb66e4dd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R3608176449fd4bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R55ef157f2b1842e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Rb7cb8cb503284a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rea635afe66464f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rd23ca5cda31c46ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R1ff96ced72544217"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rfbf36de07c7443d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Ra167cf4da3164782"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R1a733535a0454b64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R25ffa3eef0c24b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Reef36b2749684ff9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T12:31:56+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T12:50:09+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2317,7 +2317,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>46272.52217592593</x:v>
+        <x:v>46272.53482638889</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Make briefs angle-driven with current sound signals
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rea635afe66464f8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rd23ca5cda31c46ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R1ff96ced72544217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rfbf36de07c7443d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="Ra167cf4da3164782"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="R1a733535a0454b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R25ffa3eef0c24b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="Reef36b2749684ff9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R524292c26d2f4847"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R79622b088f444c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rd472848e309b4cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rf33dc233d2d643a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="R956599bb7e704b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="Rce6f5415575d4934"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R4724c709fec342ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="R7f4ab8077dcb4738"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T12:50:09+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T15:34:50+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2317,7 +2317,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>46272.53482638889</x:v>
+        <x:v>46272.649189814816</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Add routine integration and creator discovery
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,14 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R524292c26d2f4847"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R79622b088f444c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rd472848e309b4cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="4" r:id="Rf33dc233d2d643a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="5" r:id="R956599bb7e704b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="6" r:id="Rce6f5415575d4934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" r:id="R4724c709fec342ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="8" r:id="R7f4ab8077dcb4738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R60aeb95247354714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rc047b5f8ab964bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R2ce1828190494c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="4" r:id="R159bdc5fd9c948a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="5" r:id="R1451973300814919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="6" r:id="R6f2a0ff10b7f4408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="7" r:id="R01b62eb1d95249e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="R894691d66e39446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="R31428b580b9543af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="R5535c9d638914710"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
-    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd hh:mm"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -78,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -104,13 +107,75 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -335,7 +400,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T15:34:50+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T16:23:23+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1026,6 +1091,95 @@
       </x:colorScale>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Run log</x:v>
+      </x:c>
+      <x:c r="B1" s="14"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Current export metadata and definitions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="3" t="str">
+        <x:v>Generated at</x:v>
+      </x:c>
+      <x:c r="B5" s="25" t="n">
+        <x:v>46272.682905092595</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>Viral-qualified sources</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="n">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="3" t="str">
+        <x:v>Watchlist sources</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>Viral rule</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Qualified when likes &gt;= 10,000 OR views &gt;= 1,000,000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>Taxonomy</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>Campaign territory → strategic angle → hook → execution</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>Opportunity formula</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>25% momentum + 30% brand fit + 25% Q4 potential + 15% gifting relevance + 5% evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="4" t="str">
+        <x:v>Source method</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="str">
+        <x:v>Observed TikTok search metrics captured in the manual source library</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1621,6 +1775,375 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="55" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Routine integration references</x:v>
+      </x:c>
+      <x:c r="D1" s="9"/>
+      <x:c r="F1" s="9"/>
+      <x:c r="K1" s="18"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Evergreen format references are kept separate from viral evidence. Metrics are public snapshots, not forecasts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Execution</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Evidence role</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Creator</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Followers</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>US eligible</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Observed likes</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>First frame</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Story pattern</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>CoBa adaptation</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="K4" s="8" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Voice-over routine review</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Evergreen format reference — not viral proof</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>@jemaialzonia</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>29700</x:v>
+      </x:c>
+      <x:c r="E5" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>After-shaving leg routine title in a real bathroom setting</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Skin context → ordered routine steps → product integration → smoother-looking finish</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>Integrate one CoBa product into a 3–5 step low-maintenance shower or shaving routine and explain the job it performs in natural American English.</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="str">
+        <x:v>https://www.instagram.com/p/Db3gF5hhxVx/</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="36" hidden="0" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>Trendy-music routine edit</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="str">
+        <x:v>Viral execution reference — creator is not US-based</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>@sheissupra</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="n">
+        <x:v>37700</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="n">
+        <x:v>59000</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="str">
+        <x:v>Post-shower towel-wrap shot holding the routine products with a clear promise overlay</x:v>
+      </x:c>
+      <x:c r="H6" s="13" t="str">
+        <x:v>Outcome promise → fast product stack → tactile application cuts → smooth-legs payoff</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="str">
+        <x:v>Use a rising commercially cleared sound, 4–7 beat-matched close-ups and one plain-English overlay such as ‘the Vietnamese bodycare combo for smooth-looking legs.’</x:v>
+      </x:c>
+      <x:c r="J6" s="13" t="str">
+        <x:v>https://www.instagram.com/p/DbDX2Vwt3D5/</x:v>
+      </x:c>
+      <x:c r="K6" s="13" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="52" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="52" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="55" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="55" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Creator discovery</x:v>
+      </x:c>
+      <x:c r="B1" s="21"/>
+      <x:c r="G1" s="9"/>
+      <x:c r="H1" s="21"/>
+      <x:c r="I1" s="21"/>
+      <x:c r="J1" s="21"/>
+      <x:c r="K1" s="21"/>
+      <x:c r="L1" s="21"/>
+      <x:c r="R1" s="18"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Micro-creator research queue. Budget likelihood is an unconfirmed planning estimate until a creator supplies a quote.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Creator</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Handle</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Country</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Location evidence</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>Followers</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Posts audited</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>Routine fit</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
+        <x:v>Viral potential</x:v>
+      </x:c>
+      <x:c r="K4" s="8" t="str">
+        <x:v>Candid</x:v>
+      </x:c>
+      <x:c r="L4" s="8" t="str">
+        <x:v>US fit</x:v>
+      </x:c>
+      <x:c r="M4" s="8" t="str">
+        <x:v>Budget likelihood</x:v>
+      </x:c>
+      <x:c r="N4" s="8" t="str">
+        <x:v>Budget basis</x:v>
+      </x:c>
+      <x:c r="O4" s="8" t="str">
+        <x:v>Contact route</x:v>
+      </x:c>
+      <x:c r="P4" s="8" t="str">
+        <x:v>Profile</x:v>
+      </x:c>
+      <x:c r="Q4" s="8" t="str">
+        <x:v>Reference</x:v>
+      </x:c>
+      <x:c r="R4" s="8" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Needs 3-post audit</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Jemaia Alzonia</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>@jemaialzonia</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Profile states Dallas</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="n">
+        <x:v>29700</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="12" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L5" s="12" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M5" s="12" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="N5" s="12" t="str">
+        <x:v>Model estimate from follower band only; request a quote before booking</x:v>
+      </x:c>
+      <x:c r="O5" s="12" t="str">
+        <x:v>Contact route in profile bio</x:v>
+      </x:c>
+      <x:c r="P5" s="12" t="str">
+        <x:v>https://www.instagram.com/jemaialzonia/</x:v>
+      </x:c>
+      <x:c r="Q5" s="12" t="str">
+        <x:v>https://www.instagram.com/p/Db3gF5hhxVx/</x:v>
+      </x:c>
+      <x:c r="R5" s="12" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="13" t="str">
+        <x:v>Not US eligible</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>Supra</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="str">
+        <x:v>@sheissupra</x:v>
+      </x:c>
+      <x:c r="E6" s="13" t="str">
+        <x:v>Spain</x:v>
+      </x:c>
+      <x:c r="F6" s="13" t="str">
+        <x:v>Profile states Alicante</x:v>
+      </x:c>
+      <x:c r="G6" s="13" t="n">
+        <x:v>37700</x:v>
+      </x:c>
+      <x:c r="H6" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I6" s="13" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="J6" s="13" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K6" s="13" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="L6" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="13" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="N6" s="13" t="str">
+        <x:v>Model estimate from follower band only; request a quote before booking</x:v>
+      </x:c>
+      <x:c r="O6" s="13" t="str">
+        <x:v>Contact route in profile bio</x:v>
+      </x:c>
+      <x:c r="P6" s="13" t="str">
+        <x:v>https://www.instagram.com/sheissupra/</x:v>
+      </x:c>
+      <x:c r="Q6" s="13" t="str">
+        <x:v>https://www.instagram.com/p/DbDX2Vwt3D5/</x:v>
+      </x:c>
+      <x:c r="R6" s="13" t="n">
+        <x:v>46272</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="B5:B6">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
@@ -1632,7 +2155,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A1" s="15" t="str">
+      <x:c r="A1" s="24" t="str">
         <x:v>Watchlist</x:v>
       </x:c>
       <x:c r="B1" s="9"/>
@@ -1746,7 +2269,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1874,7 +2397,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2182,7 +2705,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2282,93 +2805,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="110" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Run log</x:v>
-      </x:c>
-      <x:c r="B1" s="14"/>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Current export metadata and definitions.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3"/>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Value</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="3" t="str">
-        <x:v>Generated at</x:v>
-      </x:c>
-      <x:c r="B5" s="16" t="n">
-        <x:v>46272.649189814816</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>Viral-qualified sources</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>Watchlist sources</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>Viral rule</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>Qualified when likes &gt;= 10,000 OR views &gt;= 1,000,000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="3" t="str">
-        <x:v>Taxonomy</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="str">
-        <x:v>Campaign territory → strategic angle → hook → execution</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>Opportunity formula</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str">
-        <x:v>25% momentum + 30% brand fit + 25% Q4 potential + 15% gifting relevance + 5% evidence</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="4" t="str">
-        <x:v>Source method</x:v>
-      </x:c>
-      <x:c r="B11" s="4" t="str">
-        <x:v>Observed TikTok search metrics captured in the manual source library</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Make Q4 briefs month and owner aware
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R60aeb95247354714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="Rc047b5f8ab964bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R2ce1828190494c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="4" r:id="R159bdc5fd9c948a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="5" r:id="R1451973300814919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="6" r:id="R6f2a0ff10b7f4408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Playbook" sheetId="7" r:id="R01b62eb1d95249e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="R894691d66e39446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="R31428b580b9543af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="R5535c9d638914710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R0b49fa7b062e4531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R47e4058447614e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R0ccb26303e004c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Plan" sheetId="4" r:id="Ra7dd1858856e4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="5" r:id="R4f8c28fa10034d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="6" r:id="Reeb66901399646ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="7" r:id="R5316ea00696a4f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="Rd89a4351dfd64717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="Re379b5e213bb4a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="R7a5a1f136c3d494a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -400,7 +400,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T16:23:23+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T16:45:04+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1128,7 +1128,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>46272.682905092595</x:v>
+        <x:v>46272.697962962964</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1775,6 +1775,1180 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Monthly content plan</x:v>
+      </x:c>
+      <x:c r="D1" s="9"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Planning weights and viral-potential indices for September–December. Indices prioritize tests; they are not performance forecasts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Pillar</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Opening</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Sep posts</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Sep potential</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Oct posts</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>Oct potential</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Nov posts</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>Nov potential</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
+        <x:v>Dec posts</x:v>
+      </x:c>
+      <x:c r="K4" s="8" t="str">
+        <x:v>Dec potential</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Problem → solution</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>scrub-soothe-7</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="E5" s="22" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="F5" s="22" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="H5" s="22" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="I5" s="22" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="J5" s="22" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="K5" s="22" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>Girl-math, gift closet</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>exfoliate-3</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="K6" s="22" t="n">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>Ungatekeeping, price alibi</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>exfoliate-3; scrub-soothe-7; bath-body-7</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G7" s="22" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="H7" s="22" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="K7" s="22" t="n">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Give one, keep one</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>scrub-soothe-7; bath-body-7</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="22" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F8" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G8" s="22" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H8" s="22" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K8" s="22" t="n">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" hidden="0" customHeight="1">
+      <x:c r="A9" s="13" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="str">
+        <x:v>Anti-landfill</x:v>
+      </x:c>
+      <x:c r="C9" s="13" t="str">
+        <x:v>scrub-soothe-7; bath-body-7; exfoliate-3</x:v>
+      </x:c>
+      <x:c r="D9" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F9" s="23" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="H9" s="23" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="J9" s="23" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="K9" s="23" t="n">
+        <x:v>66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="14"/>
+      <x:c r="B10" s="14"/>
+      <x:c r="C10" s="14"/>
+      <x:c r="D10" s="14"/>
+      <x:c r="E10" s="14"/>
+      <x:c r="F10" s="14"/>
+      <x:c r="G10" s="14"/>
+      <x:c r="H10" s="14"/>
+      <x:c r="I10" s="14"/>
+      <x:c r="J10" s="14"/>
+      <x:c r="K10" s="14"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Job</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>Depth</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>Focus</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:v>CTA direction</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>Operations</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="str">
+        <x:v>Blocked language</x:v>
+      </x:c>
+      <x:c r="H11" s="14"/>
+      <x:c r="I11" s="14"/>
+      <x:c r="J11" s="14"/>
+      <x:c r="K11" s="14"/>
+    </x:row>
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>Prep and seed search</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>Light gifting</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="str">
+        <x:v>Aesop Alternative plus a truthful reason to buy early</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="str">
+        <x:v>Discover the ritual early; use directional CTA only until bundles are finalized.</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="str">
+        <x:v>Send 100 TikTok samples. Basket leaves warehouse in week 4.</x:v>
+      </x:c>
+      <x:c r="G12" s="12" t="str">
+        <x:v>hostess; Secret Santa; White Elephant; occasion gift; named bundle or set</x:v>
+      </x:c>
+      <x:c r="H12" s="14"/>
+      <x:c r="I12" s="14"/>
+      <x:c r="J12" s="14"/>
+      <x:c r="K12" s="14"/>
+    </x:row>
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>Open gifting</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>Full gifting begins</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>Gift Guide, Keepsake, hostess and early occasions</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="str">
+        <x:v>Shop the gift section; explain the real value of buying multiples.</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="str">
+        <x:v>Send 100 standard samples plus 30 baskets.</x:v>
+      </x:c>
+      <x:c r="G13" s="12" t="str">
+        <x:v>fake countdown; unconfirmed price; unconfirmed set name</x:v>
+      </x:c>
+      <x:c r="H13" s="14"/>
+      <x:c r="I13" s="14"/>
+      <x:c r="J13" s="14"/>
+      <x:c r="K13" s="14"/>
+    </x:row>
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Peak gifting push</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Highest conversion pressure</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Hostess through Nov 20, volume bundles and first truthful promotion captions</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>One for them, one for me; show the real bundle math on screen.</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="str">
+        <x:v>Double Kimie's basket posts; move three posts to volume. Use real stock and promotion data only.</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="str">
+        <x:v>fake scarcity; invented inventory; unconfirmed set name or price</x:v>
+      </x:c>
+      <x:c r="H14" s="14"/>
+      <x:c r="I14" s="14"/>
+      <x:c r="J14" s="14"/>
+      <x:c r="K14" s="14"/>
+    </x:row>
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
+      <x:c r="A15" s="13" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="str">
+        <x:v>Occasion peak and shipping truth</x:v>
+      </x:c>
+      <x:c r="C15" s="13" t="str">
+        <x:v>Deadline-led</x:v>
+      </x:c>
+      <x:c r="D15" s="13" t="str">
+        <x:v>Secret Santa, White Elephant and year-end parties</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="str">
+        <x:v>Buy in multiples and order before December 18 when the confirmed shipping cutoff applies.</x:v>
+      </x:c>
+      <x:c r="F15" s="13" t="str">
+        <x:v>Everything must ship before Dec 18. Use deadline only while operationally true.</x:v>
+      </x:c>
+      <x:c r="G15" s="13" t="str">
+        <x:v>delivery promise after cutoff; fake countdown; invented low-stock claim; unconfirmed set name or price</x:v>
+      </x:c>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+      <x:c r="J15" s="14"/>
+      <x:c r="K15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="14"/>
+      <x:c r="B16" s="14"/>
+      <x:c r="C16" s="14"/>
+      <x:c r="D16" s="14"/>
+      <x:c r="E16" s="14"/>
+      <x:c r="F16" s="14"/>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+      <x:c r="J16" s="14"/>
+      <x:c r="K16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="14"/>
+      <x:c r="B17" s="14"/>
+      <x:c r="C17" s="14"/>
+      <x:c r="D17" s="14"/>
+      <x:c r="E17" s="14"/>
+      <x:c r="F17" s="14"/>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+      <x:c r="J17" s="14"/>
+      <x:c r="K17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="8" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="B18" s="8" t="str">
+        <x:v>Stream</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="str">
+        <x:v>Sep</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>Oct</x:v>
+      </x:c>
+      <x:c r="E18" s="8" t="str">
+        <x:v>Nov</x:v>
+      </x:c>
+      <x:c r="F18" s="8" t="str">
+        <x:v>Dec</x:v>
+      </x:c>
+      <x:c r="G18" s="8" t="str">
+        <x:v>Production limits</x:v>
+      </x:c>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+      <x:c r="J18" s="14"/>
+      <x:c r="K18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="36" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Arie</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>TikTok Shop + Baskets</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G19" s="12" t="str">
+        <x:v>Do not script a precise cut when only generic B-roll is guaranteed; Use QA gates for hook, format, script and hashtags</x:v>
+      </x:c>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+      <x:c r="J19" s="14"/>
+      <x:c r="K19" s="14"/>
+    </x:row>
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>Louie</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>Amazon affiliate</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G20" s="12" t="str">
+        <x:v>Aesop Alternative rises 9 → 15; Occasions rises 2 → 17; Claims and CTA must remain Amazon-compatible</x:v>
+      </x:c>
+      <x:c r="H20" s="14"/>
+      <x:c r="I20" s="14"/>
+      <x:c r="J20" s="14"/>
+      <x:c r="K20" s="14"/>
+    </x:row>
+    <x:row r="21" ht="24" hidden="0" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Kimie</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Carousel round-up</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G21" s="12" t="str">
+        <x:v>No unboxing; No texture shot; No before-and-after; No physical product handling; No CPM claim</x:v>
+      </x:c>
+      <x:c r="H21" s="14"/>
+      <x:c r="I21" s="14"/>
+      <x:c r="J21" s="14"/>
+      <x:c r="K21" s="14"/>
+    </x:row>
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
+      <x:c r="A22" s="13" t="str">
+        <x:v>New intern</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="str">
+        <x:v>Reels / integration</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D22" s="13" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E22" s="13" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F22" s="13" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G22" s="13" t="str">
+        <x:v>If role is unfilled, cap at 15 posts; Gifting round-ups grow from 5 to 13 posts</x:v>
+      </x:c>
+      <x:c r="H22" s="14"/>
+      <x:c r="I22" s="14"/>
+      <x:c r="J22" s="14"/>
+      <x:c r="K22" s="14"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="14"/>
+      <x:c r="B23" s="14"/>
+      <x:c r="C23" s="14"/>
+      <x:c r="D23" s="14"/>
+      <x:c r="E23" s="14"/>
+      <x:c r="F23" s="14"/>
+      <x:c r="G23" s="14"/>
+      <x:c r="H23" s="14"/>
+      <x:c r="I23" s="14"/>
+      <x:c r="J23" s="14"/>
+      <x:c r="K23" s="14"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="14"/>
+      <x:c r="B24" s="14"/>
+      <x:c r="C24" s="14"/>
+      <x:c r="D24" s="14"/>
+      <x:c r="E24" s="14"/>
+      <x:c r="F24" s="14"/>
+      <x:c r="G24" s="14"/>
+      <x:c r="H24" s="14"/>
+      <x:c r="I24" s="14"/>
+      <x:c r="J24" s="14"/>
+      <x:c r="K24" s="14"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="8" t="str">
+        <x:v>Hard rule</x:v>
+      </x:c>
+      <x:c r="B25" s="8" t="str">
+        <x:v>Application</x:v>
+      </x:c>
+      <x:c r="C25" s="14"/>
+      <x:c r="D25" s="14"/>
+      <x:c r="E25" s="14"/>
+      <x:c r="F25" s="14"/>
+      <x:c r="G25" s="14"/>
+      <x:c r="H25" s="14"/>
+      <x:c r="I25" s="14"/>
+      <x:c r="J25" s="14"/>
+      <x:c r="K25" s="14"/>
+    </x:row>
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="12" t="str">
+        <x:v>Never say CoBa smells like Aesop. Compare only price position, packaging and texture.</x:v>
+      </x:c>
+      <x:c r="B26" s="12" t="str">
+        <x:v>Mandatory in every generated brief and QA review</x:v>
+      </x:c>
+      <x:c r="C26" s="14"/>
+      <x:c r="D26" s="14"/>
+      <x:c r="E26" s="14"/>
+      <x:c r="F26" s="14"/>
+      <x:c r="G26" s="14"/>
+      <x:c r="H26" s="14"/>
+      <x:c r="I26" s="14"/>
+      <x:c r="J26" s="14"/>
+      <x:c r="K26" s="14"/>
+    </x:row>
+    <x:row r="27" ht="36" hidden="0" customHeight="1">
+      <x:c r="A27" s="12" t="str">
+        <x:v>Never use fake urgency. Only use the confirmed Dec 18 cutoff, truthful inventory or visible bundle math.</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="str">
+        <x:v>Mandatory in every generated brief and QA review</x:v>
+      </x:c>
+      <x:c r="C27" s="14"/>
+      <x:c r="D27" s="14"/>
+      <x:c r="E27" s="14"/>
+      <x:c r="F27" s="14"/>
+      <x:c r="G27" s="14"/>
+      <x:c r="H27" s="14"/>
+      <x:c r="I27" s="14"/>
+      <x:c r="J27" s="14"/>
+      <x:c r="K27" s="14"/>
+    </x:row>
+    <x:row r="28" ht="36" hidden="0" customHeight="1">
+      <x:c r="A28" s="13" t="str">
+        <x:v>Do not use an unconfirmed bundle or set name. Until finalized, CTA is direction rather than a quoted price or product name.</x:v>
+      </x:c>
+      <x:c r="B28" s="13" t="str">
+        <x:v>Mandatory in every generated brief and QA review</x:v>
+      </x:c>
+      <x:c r="C28" s="14"/>
+      <x:c r="D28" s="14"/>
+      <x:c r="E28" s="14"/>
+      <x:c r="F28" s="14"/>
+      <x:c r="G28" s="14"/>
+      <x:c r="H28" s="14"/>
+      <x:c r="I28" s="14"/>
+      <x:c r="J28" s="14"/>
+      <x:c r="K28" s="14"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="14"/>
+      <x:c r="B29" s="14"/>
+      <x:c r="C29" s="14"/>
+      <x:c r="D29" s="14"/>
+      <x:c r="E29" s="14"/>
+      <x:c r="F29" s="14"/>
+      <x:c r="G29" s="14"/>
+      <x:c r="H29" s="14"/>
+      <x:c r="I29" s="14"/>
+      <x:c r="J29" s="14"/>
+      <x:c r="K29" s="14"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="14"/>
+      <x:c r="B30" s="14"/>
+      <x:c r="C30" s="14"/>
+      <x:c r="D30" s="14"/>
+      <x:c r="E30" s="14"/>
+      <x:c r="F30" s="14"/>
+      <x:c r="G30" s="14"/>
+      <x:c r="H30" s="14"/>
+      <x:c r="I30" s="14"/>
+      <x:c r="J30" s="14"/>
+      <x:c r="K30" s="14"/>
+    </x:row>
+    <x:row r="31"/>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="8" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="B32" s="8" t="str">
+        <x:v>Pillar</x:v>
+      </x:c>
+      <x:c r="C32" s="8" t="str">
+        <x:v>Creator</x:v>
+      </x:c>
+      <x:c r="D32" s="8" t="str">
+        <x:v>Likes</x:v>
+      </x:c>
+      <x:c r="E32" s="8" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="F32" s="8" t="str">
+        <x:v>Reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="3" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B33" s="3" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C33" s="3" t="str">
+        <x:v>Jemaia Alzonia</x:v>
+      </x:c>
+      <x:c r="D33" s="3" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E33" s="3" t="str">
+        <x:v>Evergreen format reference — not viral proof</x:v>
+      </x:c>
+      <x:c r="F33" s="3" t="str">
+        <x:v>https://www.instagram.com/p/Db3gF5hhxVx/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="3" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>Katie</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="n">
+        <x:v>15700</x:v>
+      </x:c>
+      <x:c r="E34" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>https://www.tiktok.com/@theglowjourney/video/7425464264938376491</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="3" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B35" s="3" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="str">
+        <x:v>Carla's Vanity</x:v>
+      </x:c>
+      <x:c r="D35" s="3" t="n">
+        <x:v>14100</x:v>
+      </x:c>
+      <x:c r="E35" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F35" s="3" t="str">
+        <x:v>https://www.tiktok.com/@carlasvanity/video/7430906870174354720</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="3" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B36" s="3" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
+        <x:v>Dovey</x:v>
+      </x:c>
+      <x:c r="D36" s="3" t="n">
+        <x:v>21400</x:v>
+      </x:c>
+      <x:c r="E36" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F36" s="3" t="str">
+        <x:v>https://www.tiktok.com/@doveydaniels/photo/7444357090778303787</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="3" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
+        <x:v>Beatriz</x:v>
+      </x:c>
+      <x:c r="D37" s="3" t="n">
+        <x:v>14600</x:v>
+      </x:c>
+      <x:c r="E37" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
+        <x:v>https://www.tiktok.com/@makelifesimpler_/video/7449387997432237334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="3" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C38" s="3" t="str">
+        <x:v>Supra</x:v>
+      </x:c>
+      <x:c r="D38" s="3" t="n">
+        <x:v>59000</x:v>
+      </x:c>
+      <x:c r="E38" s="3" t="str">
+        <x:v>Viral execution reference — creator is not US-based</x:v>
+      </x:c>
+      <x:c r="F38" s="3" t="str">
+        <x:v>https://www.instagram.com/p/DbDX2Vwt3D5/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>Angie</x:v>
+      </x:c>
+      <x:c r="D39" s="3" t="n">
+        <x:v>236600</x:v>
+      </x:c>
+      <x:c r="E39" s="3" t="str">
+        <x:v>Breakout</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>https://www.tiktok.com/@lifethru.angie/video/7577422345413922066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="3" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B40" s="3" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C40" s="3" t="str">
+        <x:v>Carla's Vanity</x:v>
+      </x:c>
+      <x:c r="D40" s="3" t="n">
+        <x:v>14100</x:v>
+      </x:c>
+      <x:c r="E40" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F40" s="3" t="str">
+        <x:v>https://www.tiktok.com/@carlasvanity/video/7430906870174354720</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="3" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B41" s="3" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C41" s="3" t="str">
+        <x:v>Angie</x:v>
+      </x:c>
+      <x:c r="D41" s="3" t="n">
+        <x:v>236600</x:v>
+      </x:c>
+      <x:c r="E41" s="3" t="str">
+        <x:v>Breakout</x:v>
+      </x:c>
+      <x:c r="F41" s="3" t="str">
+        <x:v>https://www.tiktok.com/@lifethru.angie/video/7577422345413922066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="3" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B42" s="3" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C42" s="3" t="str">
+        <x:v>Beatriz</x:v>
+      </x:c>
+      <x:c r="D42" s="3" t="n">
+        <x:v>14600</x:v>
+      </x:c>
+      <x:c r="E42" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F42" s="3" t="str">
+        <x:v>https://www.tiktok.com/@makelifesimpler_/video/7449387997432237334</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B43" s="3" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C43" s="3" t="str">
+        <x:v>Anbriel Lee</x:v>
+      </x:c>
+      <x:c r="D43" s="3" t="n">
+        <x:v>13300</x:v>
+      </x:c>
+      <x:c r="E43" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F43" s="3" t="str">
+        <x:v>https://www.tiktok.com/@anbriellee/video/7652481251181448479</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B44" s="3" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C44" s="3" t="str">
+        <x:v>Chelsea</x:v>
+      </x:c>
+      <x:c r="D44" s="3" t="n">
+        <x:v>57600</x:v>
+      </x:c>
+      <x:c r="E44" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F44" s="3" t="str">
+        <x:v>https://www.tiktok.com/@chelsleebmoney/video/7442484871068536094</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B45" s="3" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C45" s="3" t="str">
+        <x:v>Angie</x:v>
+      </x:c>
+      <x:c r="D45" s="3" t="n">
+        <x:v>236600</x:v>
+      </x:c>
+      <x:c r="E45" s="3" t="str">
+        <x:v>Breakout</x:v>
+      </x:c>
+      <x:c r="F45" s="3" t="str">
+        <x:v>https://www.tiktok.com/@lifethru.angie/video/7577422345413922066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B46" s="3" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C46" s="3" t="str">
+        <x:v>Anbriel Lee</x:v>
+      </x:c>
+      <x:c r="D46" s="3" t="n">
+        <x:v>13300</x:v>
+      </x:c>
+      <x:c r="E46" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F46" s="3" t="str">
+        <x:v>https://www.tiktok.com/@anbriellee/video/7652481251181448479</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B47" s="3" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C47" s="3" t="str">
+        <x:v>Angie</x:v>
+      </x:c>
+      <x:c r="D47" s="3" t="n">
+        <x:v>236600</x:v>
+      </x:c>
+      <x:c r="E47" s="3" t="str">
+        <x:v>Breakout</x:v>
+      </x:c>
+      <x:c r="F47" s="3" t="str">
+        <x:v>https://www.tiktok.com/@lifethru.angie/video/7577422345413922066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="3" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B48" s="3" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C48" s="3" t="str">
+        <x:v>Chelsea</x:v>
+      </x:c>
+      <x:c r="D48" s="3" t="n">
+        <x:v>57600</x:v>
+      </x:c>
+      <x:c r="E48" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F48" s="3" t="str">
+        <x:v>https://www.tiktok.com/@chelsleebmoney/video/7442484871068536094</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="3" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B49" s="3" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C49" s="3" t="str">
+        <x:v>Jemaia Alzonia</x:v>
+      </x:c>
+      <x:c r="D49" s="3" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E49" s="3" t="str">
+        <x:v>Evergreen format reference — not viral proof</x:v>
+      </x:c>
+      <x:c r="F49" s="3" t="str">
+        <x:v>https://www.instagram.com/p/Db3gF5hhxVx/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="3" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B50" s="3" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C50" s="3" t="str">
+        <x:v>Chelsea</x:v>
+      </x:c>
+      <x:c r="D50" s="3" t="n">
+        <x:v>57600</x:v>
+      </x:c>
+      <x:c r="E50" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F50" s="3" t="str">
+        <x:v>https://www.tiktok.com/@chelsleebmoney/video/7442484871068536094</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="3" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B51" s="3" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C51" s="3" t="str">
+        <x:v>Carla's Vanity</x:v>
+      </x:c>
+      <x:c r="D51" s="3" t="n">
+        <x:v>14100</x:v>
+      </x:c>
+      <x:c r="E51" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F51" s="3" t="str">
+        <x:v>https://www.tiktok.com/@carlasvanity/video/7430906870174354720</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="3" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C52" s="3" t="str">
+        <x:v>Dovey</x:v>
+      </x:c>
+      <x:c r="D52" s="3" t="n">
+        <x:v>21400</x:v>
+      </x:c>
+      <x:c r="E52" s="3" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F52" s="3" t="str">
+        <x:v>https://www.tiktok.com/@doveydaniels/photo/7444357090778303787</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="4" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B53" s="4" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C53" s="4" t="str">
+        <x:v>Chelsea</x:v>
+      </x:c>
+      <x:c r="D53" s="4" t="n">
+        <x:v>57600</x:v>
+      </x:c>
+      <x:c r="E53" s="4" t="str">
+        <x:v>Qualified</x:v>
+      </x:c>
+      <x:c r="F53" s="4" t="str">
+        <x:v>https://www.tiktok.com/@chelsleebmoney/video/7442484871068536094</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="E5:K9">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E5:E9">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G5:G9">
+    <x:cfRule type="colorScale" priority="3">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I5:I9">
+    <x:cfRule type="colorScale" priority="4">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="K5:K9">
+    <x:cfRule type="colorScale" priority="5">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFF4D8D2"/>
+        <x:color rgb="FFF5E7C8"/>
+        <x:color rgb="FFD9EBDD"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
@@ -1912,7 +3086,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2140,7 +3314,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2262,134 +3436,6 @@
       </x:c>
       <x:c r="H7" s="13" t="str">
         <x:v>https://www.tiktok.com/@ashlee.alana/video/7563388481083411767</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="60" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Q4 gifting playbook</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Planning hypotheses for CoBa's Daughter based on verified viral patterns; not performance forecasts.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3"/>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>Month</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Job</x:v>
-      </x:c>
-      <x:c r="C4" s="8" t="str">
-        <x:v>Priority territory</x:v>
-      </x:c>
-      <x:c r="D4" s="8" t="str">
-        <x:v>Strategic angle</x:v>
-      </x:c>
-      <x:c r="E4" s="8" t="str">
-        <x:v>Native-US hook direction</x:v>
-      </x:c>
-      <x:c r="F4" s="8" t="str">
-        <x:v>Execution</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="12" t="str">
-        <x:v>September</x:v>
-      </x:c>
-      <x:c r="B5" s="12" t="str">
-        <x:v>Seed discovery</x:v>
-      </x:c>
-      <x:c r="C5" s="12" t="str">
-        <x:v>The Insider Edit</x:v>
-      </x:c>
-      <x:c r="D5" s="12" t="str">
-        <x:v>Be the first to edit the season's best sets</x:v>
-      </x:c>
-      <x:c r="E5" s="12" t="str">
-        <x:v>I found the bodycare gift nobody on her list has seen yet.</x:v>
-      </x:c>
-      <x:c r="F5" s="12" t="str">
-        <x:v>Talking-head edit</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="12" t="str">
-        <x:v>October</x:v>
-      </x:c>
-      <x:c r="B6" s="12" t="str">
-        <x:v>Build gifting intent</x:v>
-      </x:c>
-      <x:c r="C6" s="12" t="str">
-        <x:v>The Gift That Proves You Know Her</x:v>
-      </x:c>
-      <x:c r="D6" s="12" t="str">
-        <x:v>Build a recipient-coded ritual</x:v>
-      </x:c>
-      <x:c r="E6" s="12" t="str">
-        <x:v>I'm building a bodycare gift for the friend who notices every detail.</x:v>
-      </x:c>
-      <x:c r="F6" s="12" t="str">
-        <x:v>Build-with-me</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="12" t="str">
-        <x:v>November</x:v>
-      </x:c>
-      <x:c r="B7" s="12" t="str">
-        <x:v>Scale utility</x:v>
-      </x:c>
-      <x:c r="C7" s="12" t="str">
-        <x:v>Make the List Disappear</x:v>
-      </x:c>
-      <x:c r="D7" s="12" t="str">
-        <x:v>Abundance that solves the whole gift list</x:v>
-      </x:c>
-      <x:c r="E7" s="12" t="str">
-        <x:v>One thoughtful ritual for every hard-to-shop-for woman on my list.</x:v>
-      </x:c>
-      <x:c r="F7" s="12" t="str">
-        <x:v>Recipient roll call</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="13" t="str">
-        <x:v>December</x:v>
-      </x:c>
-      <x:c r="B8" s="13" t="str">
-        <x:v>Create desire and urgency</x:v>
-      </x:c>
-      <x:c r="C8" s="13" t="str">
-        <x:v>The Hard-to-Impress Recipient</x:v>
-      </x:c>
-      <x:c r="D8" s="13" t="str">
-        <x:v>Gift the discovery she has not seen</x:v>
-      </x:c>
-      <x:c r="E8" s="13" t="str">
-        <x:v>What do you give the woman who already has everything? This.</x:v>
-      </x:c>
-      <x:c r="F8" s="13" t="str">
-        <x:v>Talking head plus keepsake reveal</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add continuous TikTok creator scout
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="R0b49fa7b062e4531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R47e4058447614e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="R0ccb26303e004c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Plan" sheetId="4" r:id="Ra7dd1858856e4f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="5" r:id="R4f8c28fa10034d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="6" r:id="Reeb66901399646ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="7" r:id="R5316ea00696a4f85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="Rd89a4351dfd64717"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="Re379b5e213bb4a04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="R7a5a1f136c3d494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rfaa266d3706d4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R2d02df18d2d8420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rda2ef081d1c04796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Plan" sheetId="4" r:id="R7a87ad60be0d44b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="5" r:id="R8e3681e9841e4943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="6" r:id="Rca2fd5b459c54b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="7" r:id="R46528fc9601a46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="R3c3dc85499464832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="R3e81ba39ff504b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="Ra43d173fc9d44b9e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -400,7 +400,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T16:45:04+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T18:33:54+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1018,13 +1018,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="M16" s="10" t="n">
-        <x:v>51.65</x:v>
+        <x:v>51.62</x:v>
       </x:c>
       <x:c r="N16" s="10" t="n">
         <x:v>72.5</x:v>
       </x:c>
       <x:c r="O16" s="10" t="n">
-        <x:v>49.88</x:v>
+        <x:v>49.85</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
         <x:v>https://www.tiktok.com/@anbriellee/video/7652481251181448479</x:v>
@@ -1066,13 +1066,13 @@
         <x:v>47.5</x:v>
       </x:c>
       <x:c r="M17" s="11" t="n">
-        <x:v>55.87</x:v>
+        <x:v>55.74</x:v>
       </x:c>
       <x:c r="N17" s="11" t="n">
         <x:v>82.5</x:v>
       </x:c>
       <x:c r="O17" s="11" t="n">
-        <x:v>57.18</x:v>
+        <x:v>57.07</x:v>
       </x:c>
       <x:c r="P17" s="4" t="str">
         <x:v>https://www.tiktok.com/@sydlywydly/video/7673595466268937485</x:v>
@@ -1128,7 +1128,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>46272.697962962964</x:v>
+        <x:v>46272.77354166667</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1479,13 +1479,13 @@
         <x:v>13300</x:v>
       </x:c>
       <x:c r="G11" s="11" t="n">
-        <x:v>53.53</x:v>
+        <x:v>53.46</x:v>
       </x:c>
       <x:c r="H11" s="11" t="n">
         <x:v>43.75</x:v>
       </x:c>
       <x:c r="I11" s="11" t="n">
-        <x:v>53.76</x:v>
+        <x:v>53.68</x:v>
       </x:c>
       <x:c r="J11" s="11" t="n">
         <x:v>77.5</x:v>

</xml_diff>

<commit_message>
Make monthly content allocation operational
</commit_message>
<xml_diff>
--- a/outputs/viral-angle-radar.xlsx
+++ b/outputs/viral-angle-radar.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rfaa266d3706d4894"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R2d02df18d2d8420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rda2ef081d1c04796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Plan" sheetId="4" r:id="R7a87ad60be0d44b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="5" r:id="R8e3681e9841e4943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="6" r:id="Rca2fd5b459c54b25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="7" r:id="R46528fc9601a46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="8" r:id="R3c3dc85499464832"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="9" r:id="R3e81ba39ff504b0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="10" r:id="Ra43d173fc9d44b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Viral Benchmarks" sheetId="1" r:id="Rae89f4f915ac4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angle Radar" sheetId="2" r:id="R7cfc9e345b9a4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Territories" sheetId="3" r:id="Rf302013747784b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Plan" sheetId="4" r:id="Rc479664b217549ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Allocation" sheetId="5" r:id="Rf51f77ef12d5465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routine References" sheetId="6" r:id="R7579c7c0f98e4536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creator Discovery" sheetId="7" r:id="R6b739e5e8e914530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="8" r:id="R4dae32977df546ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Creators" sheetId="9" r:id="Rbaf1dd8e0efe4d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="10" r:id="R89c031869cce4f84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="11" r:id="Rf0804560035c404e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -400,7 +401,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T18:33:54+00:00.</x:v>
+        <x:v>Only posts with 10K+ likes or 1M+ views. Generated 2026-09-07T18:53:51+00:00.</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1100,6 +1101,108 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="45" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Data quality</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Qualification is independent from brand-fit scoring.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Count / rule</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="3" t="str">
+        <x:v>Viral qualification</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="str">
+        <x:v>Likes &gt;= 10,000 OR views &gt;= 1,000,000</x:v>
+      </x:c>
+      <x:c r="C5" s="3" t="str">
+        <x:v>Required before ranking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>Breakout tier</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>Likes &gt;= 100,000 OR views &gt;= 3,000,000</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="str">
+        <x:v>Use as strongest pattern signal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="3" t="str">
+        <x:v>Viral sources</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>Included in angle radar and briefs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>Watchlist</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>Excluded from viral outputs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>Missing views</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>Qualified by observed likes where available</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="4" t="str">
+        <x:v>Unverified creator country</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C10" s="4" t="str">
+        <x:v>Verify before creator outreach</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="110" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1128,7 +1231,7 @@
         <x:v>Generated at</x:v>
       </x:c>
       <x:c r="B5" s="25" t="n">
-        <x:v>46272.77354166667</x:v>
+        <x:v>46272.78739583334</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1835,7 +1938,7 @@
         <x:v>Dec potential</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>Evergreen body care</x:v>
       </x:c>
@@ -1843,7 +1946,7 @@
         <x:v>Problem → solution</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>scrub-soothe-7</x:v>
+        <x:v>exfoliate-3; scrub-soothe-7; bath-body-7</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:v>69</x:v>
@@ -1870,7 +1973,7 @@
         <x:v>90</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>The Gift Guide</x:v>
       </x:c>
@@ -1878,7 +1981,7 @@
         <x:v>Girl-math, gift closet</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>exfoliate-3</x:v>
+        <x:v>exfoliate-3; scrub-soothe-7; bath-body-7</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
         <x:v>16</x:v>
@@ -1940,7 +2043,7 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>The Keepsake</x:v>
       </x:c>
@@ -1948,7 +2051,7 @@
         <x:v>Give one, keep one</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>scrub-soothe-7; bath-body-7</x:v>
+        <x:v>exfoliate-3; scrub-soothe-7; bath-body-7</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
         <x:v>4</x:v>
@@ -1983,7 +2086,7 @@
         <x:v>Anti-landfill</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>scrub-soothe-7; bath-body-7; exfoliate-3</x:v>
+        <x:v>exfoliate-3; scrub-soothe-7; bath-body-7</x:v>
       </x:c>
       <x:c r="D9" s="13" t="n">
         <x:v>2</x:v>
@@ -2949,6 +3052,2041 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A1" s="1" t="str">
+        <x:v>Monthly content allocation</x:v>
+      </x:c>
+      <x:c r="C1" s="9"/>
+      <x:c r="D1" s="9"/>
+      <x:c r="E1" s="9"/>
+      <x:c r="F1" s="9"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Exact pieces by month, pillar, product and strategic angle. Product, angle and owner totals reconcile to monthly output.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>Pillar</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="str">
+        <x:v>Total pieces</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G4" s="14"/>
+      <x:c r="H4" s="8" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>Total pieces</x:v>
+      </x:c>
+      <x:c r="J4" s="8" t="str">
+        <x:v>Owner capacity</x:v>
+      </x:c>
+      <x:c r="K4" s="8" t="str">
+        <x:v>Reconciled</x:v>
+      </x:c>
+      <x:c r="L4" s="14"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G5" s="14"/>
+      <x:c r="H5" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K5" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L5" s="14"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="14"/>
+      <x:c r="H6" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J6" s="12" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="K6" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L6" s="14"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G7" s="14"/>
+      <x:c r="H7" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="I7" s="12" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="J7" s="12" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="K7" s="19" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L7" s="14"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="14"/>
+      <x:c r="H8" s="13" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="I8" s="13" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="J8" s="13" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="K8" s="20" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L8" s="14"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="14"/>
+      <x:c r="H9" s="14"/>
+      <x:c r="I9" s="14"/>
+      <x:c r="J9" s="14"/>
+      <x:c r="K9" s="14"/>
+      <x:c r="L9" s="14"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F10" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G10" s="14"/>
+      <x:c r="H10" s="14"/>
+      <x:c r="I10" s="14"/>
+      <x:c r="J10" s="14"/>
+      <x:c r="K10" s="14"/>
+      <x:c r="L10" s="14"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F11" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G11" s="14"/>
+      <x:c r="H11" s="8" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="I11" s="8" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="J11" s="8" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="K11" s="8" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="L11" s="8" t="str">
+        <x:v>December</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G12" s="14"/>
+      <x:c r="H12" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="I12" s="12" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J12" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K12" s="12" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="L12" s="12" t="n">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G13" s="14"/>
+      <x:c r="H13" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="I13" s="12" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="J13" s="12" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="K13" s="12" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="L13" s="12" t="n">
+        <x:v>56</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G14" s="14"/>
+      <x:c r="H14" s="13" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="I14" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J14" s="13" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="K14" s="13" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="L14" s="13" t="n">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G15" s="14"/>
+      <x:c r="H15" s="14"/>
+      <x:c r="I15" s="14"/>
+      <x:c r="J15" s="14"/>
+      <x:c r="K15" s="14"/>
+      <x:c r="L15" s="14"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G16" s="14"/>
+      <x:c r="H16" s="14"/>
+      <x:c r="I16" s="14"/>
+      <x:c r="J16" s="14"/>
+      <x:c r="K16" s="14"/>
+      <x:c r="L16" s="14"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G17" s="14"/>
+      <x:c r="H17" s="14"/>
+      <x:c r="I17" s="14"/>
+      <x:c r="J17" s="14"/>
+      <x:c r="K17" s="14"/>
+      <x:c r="L17" s="14"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G18" s="14"/>
+      <x:c r="H18" s="14"/>
+      <x:c r="I18" s="14"/>
+      <x:c r="J18" s="14"/>
+      <x:c r="K18" s="14"/>
+      <x:c r="L18" s="14"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G19" s="14"/>
+      <x:c r="H19" s="14"/>
+      <x:c r="I19" s="14"/>
+      <x:c r="J19" s="14"/>
+      <x:c r="K19" s="14"/>
+      <x:c r="L19" s="14"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G20" s="14"/>
+      <x:c r="H20" s="14"/>
+      <x:c r="I20" s="14"/>
+      <x:c r="J20" s="14"/>
+      <x:c r="K20" s="14"/>
+      <x:c r="L20" s="14"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G21" s="14"/>
+      <x:c r="H21" s="14"/>
+      <x:c r="I21" s="14"/>
+      <x:c r="J21" s="14"/>
+      <x:c r="K21" s="14"/>
+      <x:c r="L21" s="14"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C22" s="12" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G22" s="14"/>
+      <x:c r="H22" s="14"/>
+      <x:c r="I22" s="14"/>
+      <x:c r="J22" s="14"/>
+      <x:c r="K22" s="14"/>
+      <x:c r="L22" s="14"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C23" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D23" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G23" s="14"/>
+      <x:c r="H23" s="14"/>
+      <x:c r="I23" s="14"/>
+      <x:c r="J23" s="14"/>
+      <x:c r="K23" s="14"/>
+      <x:c r="L23" s="14"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="13" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D24" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E24" s="13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F24" s="13" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G24" s="14"/>
+      <x:c r="H24" s="14"/>
+      <x:c r="I24" s="14"/>
+      <x:c r="J24" s="14"/>
+      <x:c r="K24" s="14"/>
+      <x:c r="L24" s="14"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="14"/>
+      <x:c r="B25" s="14"/>
+      <x:c r="C25" s="14"/>
+      <x:c r="D25" s="14"/>
+      <x:c r="E25" s="14"/>
+      <x:c r="F25" s="14"/>
+      <x:c r="G25" s="14"/>
+      <x:c r="H25" s="14"/>
+      <x:c r="I25" s="14"/>
+      <x:c r="J25" s="14"/>
+      <x:c r="K25" s="14"/>
+      <x:c r="L25" s="14"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="14"/>
+      <x:c r="B26" s="14"/>
+      <x:c r="C26" s="14"/>
+      <x:c r="D26" s="14"/>
+      <x:c r="E26" s="14"/>
+      <x:c r="F26" s="14"/>
+      <x:c r="G26" s="14"/>
+      <x:c r="H26" s="14"/>
+      <x:c r="I26" s="14"/>
+      <x:c r="J26" s="14"/>
+      <x:c r="K26" s="14"/>
+      <x:c r="L26" s="14"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="8" t="str">
+        <x:v>Month</x:v>
+      </x:c>
+      <x:c r="B27" s="8" t="str">
+        <x:v>Pillar</x:v>
+      </x:c>
+      <x:c r="C27" s="8" t="str">
+        <x:v>Strategic angle</x:v>
+      </x:c>
+      <x:c r="D27" s="8" t="str">
+        <x:v>Pieces</x:v>
+      </x:c>
+      <x:c r="E27" s="8" t="str">
+        <x:v>Share of pillar (%)</x:v>
+      </x:c>
+      <x:c r="F27" s="8" t="str">
+        <x:v>Lead products</x:v>
+      </x:c>
+      <x:c r="G27" s="14"/>
+      <x:c r="H27" s="14"/>
+      <x:c r="I27" s="14"/>
+      <x:c r="J27" s="14"/>
+      <x:c r="K27" s="14"/>
+      <x:c r="L27" s="14"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B28" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C28" s="12" t="str">
+        <x:v>Integrate it into a real body routine</x:v>
+      </x:c>
+      <x:c r="D28" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E28" s="12" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F28" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G28" s="14"/>
+      <x:c r="H28" s="14"/>
+      <x:c r="I28" s="14"/>
+      <x:c r="J28" s="14"/>
+      <x:c r="K28" s="14"/>
+      <x:c r="L28" s="14"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D29" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E29" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G29" s="14"/>
+      <x:c r="H29" s="14"/>
+      <x:c r="I29" s="14"/>
+      <x:c r="J29" s="14"/>
+      <x:c r="K29" s="14"/>
+      <x:c r="L29" s="14"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C30" s="12" t="str">
+        <x:v>Turn products into a complete ritual</x:v>
+      </x:c>
+      <x:c r="D30" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E30" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F30" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G30" s="14"/>
+      <x:c r="H30" s="14"/>
+      <x:c r="I30" s="14"/>
+      <x:c r="J30" s="14"/>
+      <x:c r="K30" s="14"/>
+      <x:c r="L30" s="14"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C31" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D31" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E31" s="12" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F31" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G31" s="14"/>
+      <x:c r="H31" s="14"/>
+      <x:c r="I31" s="14"/>
+      <x:c r="J31" s="14"/>
+      <x:c r="K31" s="14"/>
+      <x:c r="L31" s="14"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C32" s="12" t="str">
+        <x:v>Be the first to edit the season's best sets</x:v>
+      </x:c>
+      <x:c r="D32" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E32" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F32" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G32" s="14"/>
+      <x:c r="H32" s="14"/>
+      <x:c r="I32" s="14"/>
+      <x:c r="J32" s="14"/>
+      <x:c r="K32" s="14"/>
+      <x:c r="L32" s="14"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B33" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C33" s="12" t="str">
+        <x:v>Gift the discovery she has not seen</x:v>
+      </x:c>
+      <x:c r="D33" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E33" s="12" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F33" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G33" s="14"/>
+      <x:c r="H33" s="14"/>
+      <x:c r="I33" s="14"/>
+      <x:c r="J33" s="14"/>
+      <x:c r="K33" s="14"/>
+      <x:c r="L33" s="14"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G34" s="14"/>
+      <x:c r="H34" s="14"/>
+      <x:c r="I34" s="14"/>
+      <x:c r="J34" s="14"/>
+      <x:c r="K34" s="14"/>
+      <x:c r="L34" s="14"/>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B35" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D35" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E35" s="12" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G35" s="14"/>
+      <x:c r="H35" s="14"/>
+      <x:c r="I35" s="14"/>
+      <x:c r="J35" s="14"/>
+      <x:c r="K35" s="14"/>
+      <x:c r="L35" s="14"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D36" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E36" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G36" s="14"/>
+      <x:c r="H36" s="14"/>
+      <x:c r="I36" s="14"/>
+      <x:c r="J36" s="14"/>
+      <x:c r="K36" s="14"/>
+      <x:c r="L36" s="14"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="str">
+        <x:v>Curate her aesthetic in miniature</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G37" s="14"/>
+      <x:c r="H37" s="14"/>
+      <x:c r="I37" s="14"/>
+      <x:c r="J37" s="14"/>
+      <x:c r="K37" s="14"/>
+      <x:c r="L37" s="14"/>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G38" s="14"/>
+      <x:c r="H38" s="14"/>
+      <x:c r="I38" s="14"/>
+      <x:c r="J38" s="14"/>
+      <x:c r="K38" s="14"/>
+      <x:c r="L38" s="14"/>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="12" t="str">
+        <x:v>September</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G39" s="14"/>
+      <x:c r="H39" s="14"/>
+      <x:c r="I39" s="14"/>
+      <x:c r="J39" s="14"/>
+      <x:c r="K39" s="14"/>
+      <x:c r="L39" s="14"/>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="str">
+        <x:v>Integrate it into a real body routine</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E40" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G40" s="14"/>
+      <x:c r="H40" s="14"/>
+      <x:c r="I40" s="14"/>
+      <x:c r="J40" s="14"/>
+      <x:c r="K40" s="14"/>
+      <x:c r="L40" s="14"/>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E41" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G41" s="14"/>
+      <x:c r="H41" s="14"/>
+      <x:c r="I41" s="14"/>
+      <x:c r="J41" s="14"/>
+      <x:c r="K41" s="14"/>
+      <x:c r="L41" s="14"/>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="str">
+        <x:v>Turn products into a complete ritual</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E42" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G42" s="14"/>
+      <x:c r="H42" s="14"/>
+      <x:c r="I42" s="14"/>
+      <x:c r="J42" s="14"/>
+      <x:c r="K42" s="14"/>
+      <x:c r="L42" s="14"/>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D43" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E43" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G43" s="14"/>
+      <x:c r="H43" s="14"/>
+      <x:c r="I43" s="14"/>
+      <x:c r="J43" s="14"/>
+      <x:c r="K43" s="14"/>
+      <x:c r="L43" s="14"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="str">
+        <x:v>Be the first to edit the season's best sets</x:v>
+      </x:c>
+      <x:c r="D44" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E44" s="12" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G44" s="14"/>
+      <x:c r="H44" s="14"/>
+      <x:c r="I44" s="14"/>
+      <x:c r="J44" s="14"/>
+      <x:c r="K44" s="14"/>
+      <x:c r="L44" s="14"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B45" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="str">
+        <x:v>Gift the discovery she has not seen</x:v>
+      </x:c>
+      <x:c r="D45" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E45" s="12" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F45" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G45" s="14"/>
+      <x:c r="H45" s="14"/>
+      <x:c r="I45" s="14"/>
+      <x:c r="J45" s="14"/>
+      <x:c r="K45" s="14"/>
+      <x:c r="L45" s="14"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B46" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D46" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E46" s="12" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F46" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G46" s="14"/>
+      <x:c r="H46" s="14"/>
+      <x:c r="I46" s="14"/>
+      <x:c r="J46" s="14"/>
+      <x:c r="K46" s="14"/>
+      <x:c r="L46" s="14"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D47" s="12" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E47" s="12" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G47" s="14"/>
+      <x:c r="H47" s="14"/>
+      <x:c r="I47" s="14"/>
+      <x:c r="J47" s="14"/>
+      <x:c r="K47" s="14"/>
+      <x:c r="L47" s="14"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D48" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E48" s="12" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G48" s="14"/>
+      <x:c r="H48" s="14"/>
+      <x:c r="I48" s="14"/>
+      <x:c r="J48" s="14"/>
+      <x:c r="K48" s="14"/>
+      <x:c r="L48" s="14"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str">
+        <x:v>Curate her aesthetic in miniature</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G49" s="14"/>
+      <x:c r="H49" s="14"/>
+      <x:c r="I49" s="14"/>
+      <x:c r="J49" s="14"/>
+      <x:c r="K49" s="14"/>
+      <x:c r="L49" s="14"/>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D50" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E50" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G50" s="14"/>
+      <x:c r="H50" s="14"/>
+      <x:c r="I50" s="14"/>
+      <x:c r="J50" s="14"/>
+      <x:c r="K50" s="14"/>
+      <x:c r="L50" s="14"/>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>October</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D51" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E51" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G51" s="14"/>
+      <x:c r="H51" s="14"/>
+      <x:c r="I51" s="14"/>
+      <x:c r="J51" s="14"/>
+      <x:c r="K51" s="14"/>
+      <x:c r="L51" s="14"/>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B52" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C52" s="12" t="str">
+        <x:v>Integrate it into a real body routine</x:v>
+      </x:c>
+      <x:c r="D52" s="12" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E52" s="12" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G52" s="14"/>
+      <x:c r="H52" s="14"/>
+      <x:c r="I52" s="14"/>
+      <x:c r="J52" s="14"/>
+      <x:c r="K52" s="14"/>
+      <x:c r="L52" s="14"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G53" s="14"/>
+      <x:c r="H53" s="14"/>
+      <x:c r="I53" s="14"/>
+      <x:c r="J53" s="14"/>
+      <x:c r="K53" s="14"/>
+      <x:c r="L53" s="14"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="str">
+        <x:v>Turn products into a complete ritual</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E54" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G54" s="14"/>
+      <x:c r="H54" s="14"/>
+      <x:c r="I54" s="14"/>
+      <x:c r="J54" s="14"/>
+      <x:c r="K54" s="14"/>
+      <x:c r="L54" s="14"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B55" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C55" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D55" s="12" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E55" s="12" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="F55" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G55" s="14"/>
+      <x:c r="H55" s="14"/>
+      <x:c r="I55" s="14"/>
+      <x:c r="J55" s="14"/>
+      <x:c r="K55" s="14"/>
+      <x:c r="L55" s="14"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B56" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C56" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D56" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E56" s="12" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F56" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G56" s="14"/>
+      <x:c r="H56" s="14"/>
+      <x:c r="I56" s="14"/>
+      <x:c r="J56" s="14"/>
+      <x:c r="K56" s="14"/>
+      <x:c r="L56" s="14"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B57" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C57" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D57" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E57" s="12" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F57" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G57" s="14"/>
+      <x:c r="H57" s="14"/>
+      <x:c r="I57" s="14"/>
+      <x:c r="J57" s="14"/>
+      <x:c r="K57" s="14"/>
+      <x:c r="L57" s="14"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B58" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C58" s="12" t="str">
+        <x:v>Be the first to edit the season's best sets</x:v>
+      </x:c>
+      <x:c r="D58" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G58" s="14"/>
+      <x:c r="H58" s="14"/>
+      <x:c r="I58" s="14"/>
+      <x:c r="J58" s="14"/>
+      <x:c r="K58" s="14"/>
+      <x:c r="L58" s="14"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B59" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C59" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D59" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E59" s="12" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F59" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G59" s="14"/>
+      <x:c r="H59" s="14"/>
+      <x:c r="I59" s="14"/>
+      <x:c r="J59" s="14"/>
+      <x:c r="K59" s="14"/>
+      <x:c r="L59" s="14"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B60" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C60" s="12" t="str">
+        <x:v>Gift the discovery she has not seen</x:v>
+      </x:c>
+      <x:c r="D60" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E60" s="12" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G60" s="14"/>
+      <x:c r="H60" s="14"/>
+      <x:c r="I60" s="14"/>
+      <x:c r="J60" s="14"/>
+      <x:c r="K60" s="14"/>
+      <x:c r="L60" s="14"/>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B61" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C61" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D61" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E61" s="12" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G61" s="14"/>
+      <x:c r="H61" s="14"/>
+      <x:c r="I61" s="14"/>
+      <x:c r="J61" s="14"/>
+      <x:c r="K61" s="14"/>
+      <x:c r="L61" s="14"/>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B62" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C62" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D62" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E62" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G62" s="14"/>
+      <x:c r="H62" s="14"/>
+      <x:c r="I62" s="14"/>
+      <x:c r="J62" s="14"/>
+      <x:c r="K62" s="14"/>
+      <x:c r="L62" s="14"/>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="12" t="str">
+        <x:v>November</x:v>
+      </x:c>
+      <x:c r="B63" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C63" s="12" t="str">
+        <x:v>Curate her aesthetic in miniature</x:v>
+      </x:c>
+      <x:c r="D63" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E63" s="12" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F63" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G63" s="14"/>
+      <x:c r="H63" s="14"/>
+      <x:c r="I63" s="14"/>
+      <x:c r="J63" s="14"/>
+      <x:c r="K63" s="14"/>
+      <x:c r="L63" s="14"/>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B64" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C64" s="12" t="str">
+        <x:v>Integrate it into a real body routine</x:v>
+      </x:c>
+      <x:c r="D64" s="12" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E64" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F64" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G64" s="14"/>
+      <x:c r="H64" s="14"/>
+      <x:c r="I64" s="14"/>
+      <x:c r="J64" s="14"/>
+      <x:c r="K64" s="14"/>
+      <x:c r="L64" s="14"/>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B65" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C65" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D65" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E65" s="12" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F65" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G65" s="14"/>
+      <x:c r="H65" s="14"/>
+      <x:c r="I65" s="14"/>
+      <x:c r="J65" s="14"/>
+      <x:c r="K65" s="14"/>
+      <x:c r="L65" s="14"/>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B66" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C66" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D66" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E66" s="12" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F66" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G66" s="14"/>
+      <x:c r="H66" s="14"/>
+      <x:c r="I66" s="14"/>
+      <x:c r="J66" s="14"/>
+      <x:c r="K66" s="14"/>
+      <x:c r="L66" s="14"/>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B67" s="12" t="str">
+        <x:v>Evergreen body care</x:v>
+      </x:c>
+      <x:c r="C67" s="12" t="str">
+        <x:v>Turn products into a complete ritual</x:v>
+      </x:c>
+      <x:c r="D67" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E67" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F67" s="12" t="str">
+        <x:v>Scrub &amp; Soothe 7-Piece; Exfoliate &amp; Nourish 3-Piece</x:v>
+      </x:c>
+      <x:c r="G67" s="14"/>
+      <x:c r="H67" s="14"/>
+      <x:c r="I67" s="14"/>
+      <x:c r="J67" s="14"/>
+      <x:c r="K67" s="14"/>
+      <x:c r="L67" s="14"/>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B68" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C68" s="12" t="str">
+        <x:v>Abundance that solves the whole gift list</x:v>
+      </x:c>
+      <x:c r="D68" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E68" s="12" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F68" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G68" s="14"/>
+      <x:c r="H68" s="14"/>
+      <x:c r="I68" s="14"/>
+      <x:c r="J68" s="14"/>
+      <x:c r="K68" s="14"/>
+      <x:c r="L68" s="14"/>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B69" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C69" s="12" t="str">
+        <x:v>Gift the discovery she has not seen</x:v>
+      </x:c>
+      <x:c r="D69" s="12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E69" s="12" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="F69" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G69" s="14"/>
+      <x:c r="H69" s="14"/>
+      <x:c r="I69" s="14"/>
+      <x:c r="J69" s="14"/>
+      <x:c r="K69" s="14"/>
+      <x:c r="L69" s="14"/>
+    </x:row>
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
+      <x:c r="A70" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B70" s="12" t="str">
+        <x:v>The Occasions</x:v>
+      </x:c>
+      <x:c r="C70" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D70" s="12" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E70" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F70" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G70" s="14"/>
+      <x:c r="H70" s="14"/>
+      <x:c r="I70" s="14"/>
+      <x:c r="J70" s="14"/>
+      <x:c r="K70" s="14"/>
+      <x:c r="L70" s="14"/>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B71" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C71" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D71" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E71" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F71" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G71" s="14"/>
+      <x:c r="H71" s="14"/>
+      <x:c r="I71" s="14"/>
+      <x:c r="J71" s="14"/>
+      <x:c r="K71" s="14"/>
+      <x:c r="L71" s="14"/>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B72" s="12" t="str">
+        <x:v>The Gift Guide</x:v>
+      </x:c>
+      <x:c r="C72" s="12" t="str">
+        <x:v>Be the first to edit the season's best sets</x:v>
+      </x:c>
+      <x:c r="D72" s="12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E72" s="12" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F72" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G72" s="14"/>
+      <x:c r="H72" s="14"/>
+      <x:c r="I72" s="14"/>
+      <x:c r="J72" s="14"/>
+      <x:c r="K72" s="14"/>
+      <x:c r="L72" s="14"/>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B73" s="12" t="str">
+        <x:v>The Aesop Alternative</x:v>
+      </x:c>
+      <x:c r="C73" s="12" t="str">
+        <x:v>Earn the right to recommend it as a gift</x:v>
+      </x:c>
+      <x:c r="D73" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E73" s="12" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F73" s="12" t="str">
+        <x:v>Exfoliate &amp; Nourish 3-Piece; Bath &amp; Body Gift Basket 7-Piece</x:v>
+      </x:c>
+      <x:c r="G73" s="14"/>
+      <x:c r="H73" s="14"/>
+      <x:c r="I73" s="14"/>
+      <x:c r="J73" s="14"/>
+      <x:c r="K73" s="14"/>
+      <x:c r="L73" s="14"/>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="12" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B74" s="12" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C74" s="12" t="str">
+        <x:v>Build a recipient-coded ritual</x:v>
+      </x:c>
+      <x:c r="D74" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E74" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F74" s="12" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G74" s="14"/>
+      <x:c r="H74" s="14"/>
+      <x:c r="I74" s="14"/>
+      <x:c r="J74" s="14"/>
+      <x:c r="K74" s="14"/>
+      <x:c r="L74" s="14"/>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="13" t="str">
+        <x:v>December</x:v>
+      </x:c>
+      <x:c r="B75" s="13" t="str">
+        <x:v>The Keepsake</x:v>
+      </x:c>
+      <x:c r="C75" s="13" t="str">
+        <x:v>Curate her aesthetic in miniature</x:v>
+      </x:c>
+      <x:c r="D75" s="13" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E75" s="13" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F75" s="13" t="str">
+        <x:v>Bath &amp; Body Gift Basket 7-Piece; Scrub &amp; Soothe 7-Piece</x:v>
+      </x:c>
+      <x:c r="G75" s="14"/>
+      <x:c r="H75" s="14"/>
+      <x:c r="I75" s="14"/>
+      <x:c r="J75" s="14"/>
+      <x:c r="K75" s="14"/>
+      <x:c r="L75" s="14"/>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="14"/>
+      <x:c r="B76" s="14"/>
+      <x:c r="C76" s="14"/>
+      <x:c r="D76" s="14"/>
+      <x:c r="E76" s="14"/>
+      <x:c r="F76" s="14"/>
+      <x:c r="G76" s="14"/>
+      <x:c r="H76" s="14"/>
+      <x:c r="I76" s="14"/>
+      <x:c r="J76" s="14"/>
+      <x:c r="K76" s="14"/>
+      <x:c r="L76" s="14"/>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="14"/>
+      <x:c r="B77" s="14"/>
+      <x:c r="C77" s="14"/>
+      <x:c r="D77" s="14"/>
+      <x:c r="E77" s="14"/>
+      <x:c r="F77" s="14"/>
+      <x:c r="G77" s="14"/>
+      <x:c r="H77" s="14"/>
+      <x:c r="I77" s="14"/>
+      <x:c r="J77" s="14"/>
+      <x:c r="K77" s="14"/>
+      <x:c r="L77" s="14"/>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="14"/>
+      <x:c r="B78" s="14"/>
+      <x:c r="C78" s="14"/>
+      <x:c r="D78" s="14"/>
+      <x:c r="E78" s="14"/>
+      <x:c r="F78" s="14"/>
+      <x:c r="G78" s="14"/>
+      <x:c r="H78" s="14"/>
+      <x:c r="I78" s="14"/>
+      <x:c r="J78" s="14"/>
+      <x:c r="K78" s="14"/>
+      <x:c r="L78" s="14"/>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="14"/>
+      <x:c r="B79" s="14"/>
+      <x:c r="C79" s="14"/>
+      <x:c r="D79" s="14"/>
+      <x:c r="E79" s="14"/>
+      <x:c r="F79" s="14"/>
+      <x:c r="G79" s="14"/>
+      <x:c r="H79" s="14"/>
+      <x:c r="I79" s="14"/>
+      <x:c r="J79" s="14"/>
+      <x:c r="K79" s="14"/>
+      <x:c r="L79" s="14"/>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="14"/>
+      <x:c r="B80" s="14"/>
+      <x:c r="C80" s="14"/>
+      <x:c r="D80" s="14"/>
+      <x:c r="E80" s="14"/>
+      <x:c r="F80" s="14"/>
+      <x:c r="G80" s="14"/>
+      <x:c r="H80" s="14"/>
+      <x:c r="I80" s="14"/>
+      <x:c r="J80" s="14"/>
+      <x:c r="K80" s="14"/>
+      <x:c r="L80" s="14"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
@@ -3086,7 +5224,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3314,7 +5452,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3443,7 +5581,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3749,106 +5887,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="45" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A1" s="1" t="str">
-        <x:v>Data quality</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>Qualification is independent from brand-fit scoring.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3"/>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>Check</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Count / rule</x:v>
-      </x:c>
-      <x:c r="C4" s="8" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="3" t="str">
-        <x:v>Viral qualification</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="str">
-        <x:v>Likes &gt;= 10,000 OR views &gt;= 1,000,000</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="str">
-        <x:v>Required before ranking</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>Breakout tier</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>Likes &gt;= 100,000 OR views &gt;= 3,000,000</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="str">
-        <x:v>Use as strongest pattern signal</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>Viral sources</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="str">
-        <x:v>Included in angle radar and briefs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>Watchlist</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>Excluded from viral outputs</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="3" t="str">
-        <x:v>Missing views</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C9" s="3" t="str">
-        <x:v>Qualified by observed likes where available</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="4" t="str">
-        <x:v>Unverified creator country</x:v>
-      </x:c>
-      <x:c r="B10" s="4" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C10" s="4" t="str">
-        <x:v>Verify before creator outreach</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>